<commit_message>
Subindo casos de uso corrigidos
</commit_message>
<xml_diff>
--- a/documentação/Testes/Caso de Teste/UC10 - MANTER PERFIL.xlsx
+++ b/documentação/Testes/Caso de Teste/UC10 - MANTER PERFIL.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="50">
   <si>
     <t xml:space="preserve">Caso de Teste</t>
   </si>
@@ -96,79 +96,6 @@
     <t xml:space="preserve">Alteração refletida imediatamente</t>
   </si>
   <si>
-    <t xml:space="preserve">CT03 - Validar E-mail Inválido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verificar tratamento de e-mail incorreto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Em tela de edição</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Inserir e-mail sem "@"
-2. Tentar salvar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-mail: "ana.silva"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mensagem "Formato de e-mail inválido"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alerta de exito exibido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- e-mail esta sendo atualizado sem @ e sem dominio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CT04 - Alterar Senha Válida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Testar fluxo de troca segura</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Usuário logado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Acessar "Segurança"
-2. Preencher campos
-3. Confirmar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nova senha: "S3nh@F0rt3!"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirmação e logout automático</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo não existe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- não exite o campo para alterar a senha na edição de perfil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CT05 - Tentar Senha Fraca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verificar política de complexidade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Em tela de alteração</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Inserir senha simples
-2. Tentar salvar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Senha: "123456"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mensagem "Use 8+ caracteres com números e símbolos"</t>
-  </si>
-  <si>
     <t xml:space="preserve">CT06 - Upload Foto Válida</t>
   </si>
   <si>
@@ -228,31 +155,6 @@
   </si>
   <si>
     <t xml:space="preserve">Conta marcada como inativa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CT09 - Cancelar Edições</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Validar descarte de alterações</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campos modificados</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Editar dados
-2. Clicar "Cancelar"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nome: "Ana → Ana Clara"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dados originais mantidos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Não existe um botão para cancelar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- Não existe um botão para cancelar a ação</t>
   </si>
   <si>
     <t xml:space="preserve">CT10 - Validar Campos Obrigatórios</t>
@@ -509,7 +411,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="32.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="31.44"/>
@@ -629,91 +531,91 @@
         <v>30</v>
       </c>
       <c r="H4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="B5" s="4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>39</v>
-      </c>
       <c r="H5" s="4" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="G6" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>39</v>
-      </c>
       <c r="H6" s="4" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>16</v>
@@ -722,122 +624,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.511805555555556" right="0.511805555555556" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>